<commit_message>
Update issue descriptions: add specific what-works/what-breaks evidence
Each issue now shows exactly which cases work and which fail,
with concrete input->output examples. Enables pointing to
specific test cases during walkthrough.
</commit_message>
<xml_diff>
--- a/compatibility_results.xlsx
+++ b/compatibility_results.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Tests'!$A$1:$I$136</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues'!$A$1:$F$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10722,14 +10722,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10745,15 +10746,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>What Works</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>What Breaks</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Spec Reference</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Related Tests</t>
         </is>
@@ -10767,20 +10773,31 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>Native JSON values silently dropped as sole attribute values</t>
+          <t>Native values inside arrays survive. "ex:tags": ["alpha","beta","gamma"] comes back (reordered but present).</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>Spec §2.2: "xsd:decimal, xsd:string, and xsd:boolean values **MAY** be represented using the JSON native data types number, string, and boolean" — explicit MAY keyword. Valid input, data silently lost</t>
+          <t>A native value as the SOLE value of an attribute is silently dropped. Tested all three JSON types:
+  "ex:name": "hello" (string) -&gt; entity becomes { } — attribute gone
+  "ex:count": 42 (integer) -&gt; entity becomes { } — attribute gone
+  "ex:flag": true (boolean) -&gt; entity becomes { } — attribute gone
+  "ex:amount": -99.5 (negative float) -&gt; entity becomes { } — attribute gone
+Even with xsd prefix explicitly declared (test 2.2-28), same result.
+Tests: 2.2-04 (string), 2.2-05 (int), 2.2-06 (float), 2.2-07 (bool), 2.2-08 (negative), 2.2-20 (bool false), 2.2-28 (string+xsd prefix).</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2, "MAY" keyword</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>2.2-04_native_string, 2.2-05_native_integer, 2.2-06_native_float, 2.2-07_native_boolean, 2.2-08_native_negative_number, 2.2-16_large_number, 2.2-20_native_boolean_false, 2.2-25_mixed_prov_and_custom_attrs, 2.2-28_native_string_with_xsd_prefix, 3.1.1-11_prov_type_native_string, 3.1.2-01_spec_example7, 3.1.3-01_spec_example9, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13, A.1-01_spec_example42, A.2-01_spec_example43</t>
         </is>
@@ -10794,20 +10811,29 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Native number/boolean in mixed arrays crash serializer</t>
+          <t>Array of only typed objects serialises (wrong format, but no crash). Array of only native strings also survives.</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Spec §2.2 Example 3 explicitly shows a mixed array containing typed objects and a plain integer `2` — the spec's own example causes a crash</t>
+          <t>Mix typed objects with native values in the same array — serialiser crashes.
+Input (spec's own Example 3): "ex:tag": [{"$":"hello","type":"xsd:string"}, 2, {"$":"Qk0=","type":"xsd:base64Binary"}]
+Result: SERIALIZE_FAILED — JsonMappingException: unknown value type null
+ProvToolbox reads the mixed array fine. It crashes only when trying to write it back. The serialiser doesn't know how to handle the native value it already parsed.
+Also crashes: 2.2-12 (typed+native bool), 2.2-22 (array of native ints [1,2,3]).</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2, Example 3</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>2.2-03_spec_example3_mixed_array, 2.2-12_mixed_typed_native_array, 2.2-22_native_int_array</t>
         </is>
@@ -10821,20 +10847,34 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>`prov:value` loses its data content on round-trip</t>
+          <t>The prov:value KEY survives in output. The type name sometimes survives.</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>`prov:value` is a defined PROV-DM attribute; data read in successfully but not written back out</t>
+          <t>The actual DATA CONTENT (the "$" value) is dropped.
+  Input: "prov:value": {"$":"42", "type":"xsd:int"}
+  Output: "prov:value": ["xsd:int"]  — "42" is gone
+  Input: "prov:value": {"$":"some text content", "type":"xsd:string"}
+  Output: "prov:value": ["xsd:string"]  — text content gone
+Inconsistency: test 3.1.1-18 (no prefix for type) — the VALUE survives but TYPE is dropped:
+  Input: {"$":"the actual content", "type":"xsd:string"}
+  Output: ["the actual content"]  — type gone, value kept
+On agents and activities it is even worse — entire prov:value disappears (see D3.1.2-1).
+Tests: 2.2-15, 2.2-23, 3.1.1-18, 3.1.1-22.</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>PROV-DM attribute definition</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>2.2-15_prov_value_typed, 2.2-23_prov_value_xsd_string, 3.1.1-18_prov_value_only</t>
         </is>
@@ -10848,20 +10888,23 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>JSON `null` as attribute value crashes parser (NPE)</t>
-        </is>
-      </c>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr"/>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>`null` is not a defined PROV-JSON value type, so rejection is correct, but the parser crashes with an unhandled NullPointerException rather than a clean parse error</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr"/>
+          <t>null is not a valid PROV-JSON value type, so rejection is correct.
+WHAT BREAKS: Instead of a clean error message like "invalid value type at line X", the parser crashes with an unhandled NullPointerException.
+This test passes our suite (we expected PARSE_FAILED), but the crash quality is the issue — any robust parser should give a meaningful error, not an unhandled NPE.</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Defensive error handling</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -10871,20 +10914,33 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Bundle deserialization completely broken — NPE crash on all bundle inputs</t>
+          <t>Nothing. 6 out of 6 bundle tests crash. Also A.3-01 (spec Example 44 with bundle).</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Spec §3.3 defines bundles with multiple examples (Examples 40–41); every bundle test crashes with NullPointerException</t>
+          <t>Every bundle, no matter how simple:
+  3.3-01: Minimal bundle (one entity inside) -&gt; NPE
+  3.3-02: Bundle with a relation -&gt; NPE
+  3.3-03: Top-level statements + bundle -&gt; NPE
+  3.3-04: Multiple bundles -&gt; NPE
+  3.3-05: Empty bundle (no statements) -&gt; NPE
+  3.3-06: Bundle with own prefix section -&gt; NPE
+All crash with: NullPointerException: Cannot invoke "QualifiedName.getPrefix()" because "this.id" is null
+The deserialiser fails to set the bundle's id field before Jackson tries to call getPrefix() on it.</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Spec Section 3.3, Examples 40-41</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>3.3-01_minimal_bundle, 3.3-02_bundle_with_relation, 3.3-03_toplevel_plus_bundle, 3.3-04_multiple_bundles, 3.3-05_empty_bundle, 3.3-06_bundle_with_prefix, A.3-01_spec_example44_simplified</t>
         </is>
@@ -10898,20 +10954,30 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>PROV-Dictionary extensions not recognized in JSON format</t>
+          <t>All standard PROV relations (wasGeneratedBy, used, wasDerivedFrom, etc.) parse fine.</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Spec Appendix B defines `hadDictionaryMember`, `derivedByInsertionFrom`, `derivedByRemovalFrom` with Examples 46–52; all dictionary data silently discarded on round-trip</t>
+          <t>The three dictionary-specific relation types from Appendix B:
+  hadDictionaryMember    (Example 46) -&gt; UnrecognizedPropertyException
+  derivedByInsertionFrom (Example 48) -&gt; UnrecognizedPropertyException
+  derivedByRemovalFrom   (Example 52) -&gt; UnrecognizedPropertyException
+The error message lists all 23 fields the deserialiser DOES recognise — dictionary types are not among them. The SortedDocument class simply has no fields for dictionary operations.
+Tests: B.1-01, B.2-01, B.3-01.</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Spec Appendix B, Examples 46-52</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>B.1-01_spec_example46, B.2-01_spec_example48, B.3-01_spec_example52</t>
         </is>
@@ -10925,20 +10991,28 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>User `_` prefix silently overridden by internal blank node mapping</t>
+          <t>All other user-defined prefixes ("ex", "custom", "myprefix") are preserved fine.</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Spec §2.1 defines `_:` for blank node identifiers per Turtle nodeID production; a user-defined `_` namespace prefix is silently overwritten without warning</t>
+          <t>Only the "_" prefix specifically.
+  Input prefix: "_": "http://example.org/my-blanks/"
+  Output: the "_" prefix is gone entirely — not in the prefix section at all
+ProvToolbox internally uses "_:" for blank nodes (per spec), but instead of co-existing with a user's "_" prefix, it overwrites it silently. No warning, no error.</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>2.1-12_user_underscore_prefix</t>
         </is>
@@ -10952,20 +11026,34 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Typed values serialized as 2-element arrays instead of `{"$":..., "type":...}`</t>
+          <t>The data content and type name both survive (usually).</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>Spec §2.2: "The value of a literal is stored in the object's special property `$`... the data type in the `type` property" — spec defines an object format; ProvToolbox outputs `[value, type]` arrays instead</t>
+          <t>The FORMAT is wrong. Spec defines typed values as JSON objects; ProvToolbox outputs 2-element arrays.
+  Spec format:     {"$": "1034", "type": "xsd:positiveInteger"}
+  ProvToolbox out: ["xsd:positiveInteger", "1034"]
+  Spec format:     {"$": "36.6", "type": "xsd:float"}
+  ProvToolbox out: ["xsd:float", "36.6"]
+  Spec format:     {"$": "Londres", "lang": "fr"}
+  ProvToolbox out: ["Londres", "fr"]
+The lang-tagged case also becomes an array — so there is no way to distinguish a language tag from a type in ProvToolbox's output.
+Any other spec-compliant tool reading this output will fail to parse typed values.
+Affects almost every test with typed attributes (60+ tests).</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2, "$" and "type" properties</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>2.2-01_spec_example1_typed, 2.2-02_lang_tagged_string, 2.2-09_single_typed_custom_attr, 2.2-13_prov_type_qualified_name, 2.2-14_prov_location_typed, 2.2-17_empty_string_value, 2.2-18_custom_type, 2.2-24_prov_label_single_lang, 2.2-25_mixed_prov_and_custom_attrs, 2.2-27_typed_xsd_string_vs_native, 3.1.1-04_all_prov_attrs, 3.1.1-05_many_custom_attrs, 3.1.1-06_collection_entity, 3.1.1-09_long_entity_id, 3.1.1-10_entity_with_activity_agent, 3.1.1-17_two_prov_types, 3.1.1-19_prov_type_typed_string, 3.1.1-21_entity_only_no_other_sections, 3.1.2-02_agent_typed_attrs, 3.1.2-04_agent_prov_label, 3.1.2-05_agent_prov_location, 3.1.2-09_agent_plus_entity, 3.1.2-15_agent_label_lang, 3.1.3-02_activity_typed_attrs, 3.1.3-05_no_times, 3.1.3-09_all_three_elements, 3.2.1-02_generation_typed_prenorm, 3.2.1-05_generation_prov_role, 3.2.1-07_no_time, 3.2.1-09_full_provenance, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time, 3.2.7-03_revision_type, 3.2.9-03_with_role, A.1-01_spec_example42, A.2-01_spec_example43</t>
         </is>
@@ -10979,20 +11067,30 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Native strings behave differently depending on context — dropped when alone, kept in arrays</t>
+          <t>Native strings in an array survive:
+  Input:  "ex:tags": ["alpha", "beta", "gamma"]
+  Output: "ex:tags": ["beta", "alpha", "gamma"]  — present but reordered</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Spec §2.2 allows native types equally in both contexts; inconsistent handling</t>
+          <t>A native string as sole value is dropped (D2.2-2):
+  Input:  "ex:name": "hello"
+  Output: entity becomes { }  — attribute gone
+Same data type, same spec permission. The only difference is whether it is the sole value or one of many in an array.</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>2.2-19_native_string_array</t>
         </is>
@@ -11006,20 +11104,24 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>2-element array output has non-deterministic element order</t>
-        </is>
-      </c>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr"/>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>The `[value, type]` arrays from D2.2-1 have unpredictable element order depending on Java hash codes, making the already-incorrect format additionally unreliable</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr"/>
+          <t>The [value, type] arrays from D2.2-1 do not have consistent element order. From the SAME test, SAME entity:
+  "ex:byteSize"    -&gt; ["xsd:positiveInteger", "1034"]     (type first)
+  "ex:compression" -&gt; ["82.5e-2", "xsd:double"]           (value first)
+The order depends on Java's internal hash codes for the strings. So a consumer cannot even rely on position to tell value from type.</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -11029,20 +11131,34 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>`prov:value` completely dropped on Agent elements</t>
+          <t>On entities, prov:value partially works (key survives, content often lost — see D2.2-5).</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>`prov:value` is a defined PROV-DM attribute for elements; read in but not written back out on agents specifically</t>
+          <t>On agents and activities, the ENTIRE prov:value attribute disappears:
+  Entity input:   "prov:value": {"$":"42","type":"xsd:int"}
+  Entity output:  "prov:value": ["xsd:int"]  — key survives, content lost
+  Agent input:    "prov:value": {"$":"agent-data-123","type":"xsd:string"}
+  Agent output:   "ex:ag1": { }  — ENTIRE attribute gone
+  Agent input:    "prov:value": {"$":"42","type":"xsd:int"}
+  Agent output:   "ex:ag1": { }  — ENTIRE attribute gone
+  Activity input: "prov:value": {"$":"computation-result","type":"xsd:string"}
+  Activity output: "ex:a1": { }  — ENTIRE attribute gone
+Tests: 3.1.2-06, 3.1.2-13 (agents), 3.1.3-07 (activity).</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>PROV-DM attribute definition</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>3.1.2-06_agent_prov_value, 3.1.2-13_agent_prov_value_int, 3.1.3-07_activity_prov_value</t>
         </is>
@@ -11056,20 +11172,28 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Multi-value `xsd:string` attributes lose type annotation</t>
+          <t>A single typed value on an agent keeps its type (as wrong array format).</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>When an agent has ≥2 `xsd:string` typed values, the type information is stripped from the output; values survive but lose their type</t>
+          <t>Two or more xsd:string values on the same attribute — type stripped:
+  Input:  "ex:role": [{"$":"developer","type":"xsd:string"}, {"$":"manager","type":"xsd:string"}]
+  Output: "ex:role": ["developer", "manager"]
+Values survive. Type annotations gone. You cannot tell if these were typed xsd:string or plain native strings.</t>
         </is>
       </c>
       <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>3.1.2-10_agent_multivalue_attr</t>
         </is>
@@ -11083,20 +11207,31 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Timestamps silently modified — timezone injected, milliseconds added, sub-ms truncated</t>
+          <t>Pre-formatted timestamps matching ProvToolbox's own output format round-trip perfectly. Test 3.1.3-13 passes with "2011-11-16T16:05:00.000+01:00".</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>Spec §3.1.3: timestamps "**MUST** conform to xsd:dateTime" — the spec does not explicitly require preserving the exact lexical form. However, injecting `+00:00` changes semantic meaning: a timezone-unspecified value becomes explicitly UTC. Spec Example 9 shows timestamps without timezone or milliseconds</t>
+          <t>Any other valid xsd:dateTime format is modified:
+  "2011-11-16T16:05:00"        -&gt; "2011-11-16T16:05:00.000+01:00"  (added .000 and local TZ)
+  "2011-11-16T16:05:00Z"       -&gt; "2011-11-16T16:05:00.000Z"       (added .000)
+  "2011-11-16T16:06:00.456789Z"-&gt; "2011-11-16T16:06:00.456Z"       (truncated microseconds)
+  "2011-11-16" (date only)     -&gt; "2011-11-16T00:00:00.000+01:00"  (added time, ms, local TZ)
+The +01:00 is the MACHINE'S LOCAL TIMEZONE — same input produces different output depending on where you run it. Adding a timezone changes semantic meaning: "unspecified timezone" becomes "explicitly UTC+1".
+Tests: 3.1.3-01 through 3.1.3-12 (except 3.1.3-13 which passes), 3.1.3-14.</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Spec Section 3.1.3, Example 9</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>3.1.3-01_spec_example9, 3.1.3-02_activity_typed_attrs, 3.1.3-03_start_time_only, 3.1.3-04_end_time_only, 3.1.3-06_multiple_activities, 3.1.3-09_all_three_elements, 3.1.3-10_time_precision, 3.1.3-14_time_date_only, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13</t>
         </is>
@@ -11110,20 +11245,28 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>Multi-value array order not preserved</t>
+          <t>Single values stay in place.</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Spec §2.2: multiple values "**MUST** be... collated in to a JSON array." Array order is semantically significant in JSON, but the spec does not explicitly require preserving it</t>
+          <t>Multi-value arrays get reordered:
+  Input:  ["alpha", "beta", "gamma"]
+  Output: ["beta", "alpha", "gamma"]
+Content survives, order does not. Array order is semantically significant in JSON, but the spec does not explicitly require preserving it.</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Spec Section 2.2</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>2.2-10_array_typed_values, 2.2-11_multiple_lang_tags, 3.1.1-13_multiple_prov_types, 3.1.2-14_agent_multivalue_qname</t>
         </is>
@@ -11137,20 +11280,28 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Element order within sections not preserved</t>
+          <t>Data within each element is complete.</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>JSON object key order is not guaranteed by the JSON specification; however many systems depend on it in practice</t>
+          <t>Element ordering within sections changes:
+  Input order:  "ex:e1", "ex:e2", "ex:e3"
+  Output order: may become "ex:e3", "ex:e1", "ex:e2"
+JSON object key order is not guaranteed by the JSON spec, so this is debatable, but many systems depend on it in practice.</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>JSON specification</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>3.1.1-03_multiple_entities, 3.1.2-03_multiple_agents, 3.1.3-06_multiple_activities, 3.2.1-08_multiple_generations</t>
         </is>
@@ -11164,20 +11315,21 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>Duplicate JSON keys — last wins silently</t>
-        </is>
-      </c>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Standard JSON parser behaviour per RFC 8259; not specific to ProvToolbox</t>
+          <t>Duplicate JSON keys in the same object — last one wins silently. This is standard JSON parser behaviour per RFC 8259, not specific to ProvToolbox.</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>RFC 8259</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>3.1.1-08_duplicate_entity_id</t>
         </is>
@@ -11191,20 +11343,25 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>`prov:role` silently dropped on elements</t>
+          <t>prov:role on relations (wasGeneratedBy, wasAssociatedWith, etc.) is preserved. Test 3.2.1-05 and 3.2.9-03 show prov:role surviving on relations (wrong array format, but data is there).</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>PROV-DM defines `prov:role` for relations, not elements. Elements can have arbitrary additional attributes, so `prov:role` should be preserved as a generic attribute, but it is not a standard element attribute</t>
+          <t>prov:role on elements (entity, agent, activity) is dropped. PROV-DM defines prov:role for relations, not elements, so dropping it on elements is arguably correct — but it could be preserved as a generic attribute.</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>PROV-DM</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>3.1.1-04_all_prov_attrs, 3.1.1-20_prov_role, 3.1.2-07_agent_prov_role, 3.1.3-08_activity_prov_role</t>
         </is>
@@ -11218,20 +11375,25 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Empty statement sections dropped from output</t>
+          <t>Sections with actual data are always present.</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Spec shows sections containing data; it does not explicitly require preserving empty sections. No data loss</t>
+          <t>Empty sections like "entity": {} are dropped from output entirely. No data was in them, so no data is lost. Cosmetic difference only.</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Spec examples</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>3.1.1-12_empty_entity_section, 3.1.2-08_empty_agent_section, 3.1.3-11_empty_activity_section, 3.2.1-10_empty_wgb_section</t>
         </is>
@@ -11245,27 +11407,28 @@
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>Property order within relation objects changed from input</t>
-        </is>
-      </c>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr"/>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>JSON object key order is not guaranteed; data intact but structure differs</t>
+          <t>Property order within relation objects is changed from input. For example, "prov:entity" and "prov:activity" keys may swap positions. JSON object key order is not guaranteed. Data is intact, only structure differs.</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
+          <t>JSON specification</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
           <t>3.2.2-01_spec_example13, 3.2.2-02_named_minimal, 3.2.2-03_anonymous_blank_node, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add workarounds column to issue reports based on source code analysis
Read ProvToolbox serialiser/deserialiser source to identify root causes
for all 19 issues and developed practical workarounds for each.

Key findings from source:
- JSON_Entity.java: @JsonIgnore on getValue() causes prov:value loss
- SortedBundle.java: hardcoded "_" prefix, empty dictionary cases
- CustomAttributeSetDeserializer: native values lost via textValue()
- SortedBundle.toBundle(): NPE on bundle id causes all bundle crashes
</commit_message>
<xml_diff>
--- a/compatibility_results.xlsx
+++ b/compatibility_results.xlsx
@@ -10727,10 +10727,10 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10746,22 +10746,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>What Works</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What Breaks</t>
+          <t>Spec Reference</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Spec Reference</t>
+          <t>Related Tests</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Related Tests</t>
+          <t>Workaround</t>
         </is>
       </c>
     </row>
@@ -10773,33 +10773,27 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>Native values inside arrays survive. "ex:tags": ["alpha","beta","gamma"] comes back (reordered but present).</t>
+          <t>Native JSON values silently dropped as sole attribute values</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>A native value as the SOLE value of an attribute is silently dropped. Tested all three JSON types:
-  "ex:name": "hello" (string) -&gt; entity becomes { } — attribute gone
-  "ex:count": 42 (integer) -&gt; entity becomes { } — attribute gone
-  "ex:flag": true (boolean) -&gt; entity becomes { } — attribute gone
-  "ex:amount": -99.5 (negative float) -&gt; entity becomes { } — attribute gone
-Even with xsd prefix explicitly declared (test 2.2-28), same result.
-Tests: 2.2-04 (string), 2.2-05 (int), 2.2-06 (float), 2.2-07 (bool), 2.2-08 (negative), 2.2-20 (bool false), 2.2-28 (string+xsd prefix).</t>
+          <t>Spec §2.2: "xsd:decimal, xsd:string, and xsd:boolean values **MAY** be represented using the JSON native data types number, string, and boolean" — explicit MAY keyword. Valid input, data silently lost</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>Spec Section 2.2, "MAY" keyword</t>
+          <t>2.2-04_native_string, 2.2-05_native_integer, 2.2-06_native_float, 2.2-07_native_boolean, 2.2-08_native_negative_number, 2.2-16_large_number, 2.2-20_native_boolean_false, 2.2-25_mixed_prov_and_custom_attrs, 2.2-28_native_string_with_xsd_prefix, 3.1.1-11_prov_type_native_string, 3.1.2-01_spec_example7, 3.1.3-01_spec_example9, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13, A.1-01_spec_example42, A.2-01_spec_example43</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>2.2-04_native_string, 2.2-05_native_integer, 2.2-06_native_float, 2.2-07_native_boolean, 2.2-08_native_negative_number, 2.2-16_large_number, 2.2-20_native_boolean_false, 2.2-25_mixed_prov_and_custom_attrs, 2.2-28_native_string_with_xsd_prefix, 3.1.1-11_prov_type_native_string, 3.1.2-01_spec_example7, 3.1.3-01_spec_example9, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13, A.1-01_spec_example42, A.2-01_spec_example43</t>
+          <t>PRE-PROCESS INPUT: Convert native JSON values to typed format. "ex:name": "hello" -&gt; "ex:name": [{"$": "hello", "type": "xsd:string"}]</t>
         </is>
       </c>
     </row>
@@ -10811,31 +10805,27 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Array of only typed objects serialises (wrong format, but no crash). Array of only native strings also survives.</t>
+          <t>Native number/boolean in mixed arrays crash serializer</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Mix typed objects with native values in the same array — serialiser crashes.
-Input (spec's own Example 3): "ex:tag": [{"$":"hello","type":"xsd:string"}, 2, {"$":"Qk0=","type":"xsd:base64Binary"}]
-Result: SERIALIZE_FAILED — JsonMappingException: unknown value type null
-ProvToolbox reads the mixed array fine. It crashes only when trying to write it back. The serialiser doesn't know how to handle the native value it already parsed.
-Also crashes: 2.2-12 (typed+native bool), 2.2-22 (array of native ints [1,2,3]).</t>
+          <t>Spec §2.2 Example 3 explicitly shows a mixed array containing typed objects and a plain integer `2` — the spec's own example causes a crash</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>Spec Section 2.2, Example 3</t>
+          <t>2.2-03_spec_example3_mixed_array, 2.2-12_mixed_typed_native_array, 2.2-22_native_int_array</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>2.2-03_spec_example3_mixed_array, 2.2-12_mixed_typed_native_array, 2.2-22_native_int_array</t>
+          <t>PRE-PROCESS INPUT: Convert native values in arrays to typed format. Eliminates the crash.</t>
         </is>
       </c>
     </row>
@@ -10847,36 +10837,27 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>The prov:value KEY survives in output. The type name sometimes survives.</t>
+          <t>`prov:value` loses its data content on round-trip</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>The actual DATA CONTENT (the "$" value) is dropped.
-  Input: "prov:value": {"$":"42", "type":"xsd:int"}
-  Output: "prov:value": ["xsd:int"]  — "42" is gone
-  Input: "prov:value": {"$":"some text content", "type":"xsd:string"}
-  Output: "prov:value": ["xsd:string"]  — text content gone
-Inconsistency: test 3.1.1-18 (no prefix for type) — the VALUE survives but TYPE is dropped:
-  Input: {"$":"the actual content", "type":"xsd:string"}
-  Output: ["the actual content"]  — type gone, value kept
-On agents and activities it is even worse — entire prov:value disappears (see D3.1.2-1).
-Tests: 2.2-15, 2.2-23, 3.1.1-18, 3.1.1-22.</t>
+          <t>`prov:value` is a defined PROV-DM attribute; data read in successfully but not written back out</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>PROV-DM attribute definition</t>
+          <t>2.2-15_prov_value_typed, 2.2-23_prov_value_xsd_string, 3.1.1-18_prov_value_only</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>2.2-15_prov_value_typed, 2.2-23_prov_value_xsd_string, 3.1.1-18_prov_value_only</t>
+          <t>PRE-PROCESS: Rename "prov:value" to custom attribute (e.g., "ex:provValue"). POST-PROCESS: Rename back.</t>
         </is>
       </c>
     </row>
@@ -10888,23 +10869,25 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr"/>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>JSON `null` as attribute value crashes parser (NPE)</t>
+        </is>
+      </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>null is not a valid PROV-JSON value type, so rejection is correct.
-WHAT BREAKS: Instead of a clean error message like "invalid value type at line X", the parser crashes with an unhandled NullPointerException.
-This test passes our suite (we expected PARSE_FAILED), but the crash quality is the issue — any robust parser should give a meaningful error, not an unhandled NPE.</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>Defensive error handling</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="inlineStr"/>
+          <t>`null` is not a defined PROV-JSON value type, so rejection is correct, but the parser crashes with an unhandled NullPointerException rather than a clean parse error</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr"/>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>PRE-PROCESS: Validate JSON and remove/replace null attribute values before passing to ProvToolbox.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -10914,35 +10897,27 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Nothing. 6 out of 6 bundle tests crash. Also A.3-01 (spec Example 44 with bundle).</t>
+          <t>Bundle deserialization completely broken — NPE crash on all bundle inputs</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Every bundle, no matter how simple:
-  3.3-01: Minimal bundle (one entity inside) -&gt; NPE
-  3.3-02: Bundle with a relation -&gt; NPE
-  3.3-03: Top-level statements + bundle -&gt; NPE
-  3.3-04: Multiple bundles -&gt; NPE
-  3.3-05: Empty bundle (no statements) -&gt; NPE
-  3.3-06: Bundle with own prefix section -&gt; NPE
-All crash with: NullPointerException: Cannot invoke "QualifiedName.getPrefix()" because "this.id" is null
-The deserialiser fails to set the bundle's id field before Jackson tries to call getPrefix() on it.</t>
+          <t>Spec §3.3 defines bundles with multiple examples (Examples 40–41); every bundle test crashes with NullPointerException</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Spec Section 3.3, Examples 40-41</t>
+          <t>3.3-01_minimal_bundle, 3.3-02_bundle_with_relation, 3.3-03_toplevel_plus_bundle, 3.3-04_multiple_bundles, 3.3-05_empty_bundle, 3.3-06_bundle_with_prefix, A.3-01_spec_example44_simplified</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>3.3-01_minimal_bundle, 3.3-02_bundle_with_relation, 3.3-03_toplevel_plus_bundle, 3.3-04_multiple_bundles, 3.3-05_empty_bundle, 3.3-06_bundle_with_prefix, A.3-01_spec_example44_simplified</t>
+          <t>NO IN-FORMAT WORKAROUND. Extract bundle contents into separate documents, or use PROV-N format.</t>
         </is>
       </c>
     </row>
@@ -10954,32 +10929,27 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>All standard PROV relations (wasGeneratedBy, used, wasDerivedFrom, etc.) parse fine.</t>
+          <t>PROV-Dictionary extensions not recognized in JSON format</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>The three dictionary-specific relation types from Appendix B:
-  hadDictionaryMember    (Example 46) -&gt; UnrecognizedPropertyException
-  derivedByInsertionFrom (Example 48) -&gt; UnrecognizedPropertyException
-  derivedByRemovalFrom   (Example 52) -&gt; UnrecognizedPropertyException
-The error message lists all 23 fields the deserialiser DOES recognise — dictionary types are not among them. The SortedDocument class simply has no fields for dictionary operations.
-Tests: B.1-01, B.2-01, B.3-01.</t>
+          <t>Spec Appendix B defines `hadDictionaryMember`, `derivedByInsertionFrom`, `derivedByRemovalFrom` with Examples 46–52; all dictionary data silently discarded on round-trip</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Spec Appendix B, Examples 46-52</t>
+          <t>B.1-01_spec_example46, B.2-01_spec_example48, B.3-01_spec_example52</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>B.1-01_spec_example46, B.2-01_spec_example48, B.3-01_spec_example52</t>
+          <t>NO IN-FORMAT WORKAROUND. Model as regular entities or use PROV-N format.</t>
         </is>
       </c>
     </row>
@@ -10991,30 +10961,27 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>All other user-defined prefixes ("ex", "custom", "myprefix") are preserved fine.</t>
+          <t>User `_` prefix silently overridden by internal blank node mapping</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Only the "_" prefix specifically.
-  Input prefix: "_": "http://example.org/my-blanks/"
-  Output: the "_" prefix is gone entirely — not in the prefix section at all
-ProvToolbox internally uses "_:" for blank nodes (per spec), but instead of co-existing with a user's "_" prefix, it overwrites it silently. No warning, no error.</t>
+          <t>Spec §2.1 defines `_:` for blank node identifiers per Turtle nodeID production; a user-defined `_` namespace prefix is silently overwritten without warning</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Spec Section 2.1</t>
+          <t>2.1-12_user_underscore_prefix</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>2.1-12_user_underscore_prefix</t>
+          <t>PRE-PROCESS: Avoid "_" as namespace prefix. Rename to "u" or "bnk" in prefix section and all qualified names.</t>
         </is>
       </c>
     </row>
@@ -11026,36 +10993,27 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>The data content and type name both survive (usually).</t>
+          <t>Typed values serialized as 2-element arrays instead of `{"$":..., "type":...}`</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>The FORMAT is wrong. Spec defines typed values as JSON objects; ProvToolbox outputs 2-element arrays.
-  Spec format:     {"$": "1034", "type": "xsd:positiveInteger"}
-  ProvToolbox out: ["xsd:positiveInteger", "1034"]
-  Spec format:     {"$": "36.6", "type": "xsd:float"}
-  ProvToolbox out: ["xsd:float", "36.6"]
-  Spec format:     {"$": "Londres", "lang": "fr"}
-  ProvToolbox out: ["Londres", "fr"]
-The lang-tagged case also becomes an array — so there is no way to distinguish a language tag from a type in ProvToolbox's output.
-Any other spec-compliant tool reading this output will fail to parse typed values.
-Affects almost every test with typed attributes (60+ tests).</t>
+          <t>Spec §2.2: "The value of a literal is stored in the object's special property `$`... the data type in the `type` property" — spec defines an object format; ProvToolbox outputs `[value, type]` arrays instead</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Spec Section 2.2, "$" and "type" properties</t>
+          <t>2.2-01_spec_example1_typed, 2.2-02_lang_tagged_string, 2.2-09_single_typed_custom_attr, 2.2-13_prov_type_qualified_name, 2.2-14_prov_location_typed, 2.2-17_empty_string_value, 2.2-18_custom_type, 2.2-24_prov_label_single_lang, 2.2-25_mixed_prov_and_custom_attrs, 2.2-27_typed_xsd_string_vs_native, 3.1.1-04_all_prov_attrs, 3.1.1-05_many_custom_attrs, 3.1.1-06_collection_entity, 3.1.1-09_long_entity_id, 3.1.1-10_entity_with_activity_agent, 3.1.1-17_two_prov_types, 3.1.1-19_prov_type_typed_string, 3.1.1-21_entity_only_no_other_sections, 3.1.2-02_agent_typed_attrs, 3.1.2-04_agent_prov_label, 3.1.2-05_agent_prov_location, 3.1.2-09_agent_plus_entity, 3.1.2-15_agent_label_lang, 3.1.3-02_activity_typed_attrs, 3.1.3-05_no_times, 3.1.3-09_all_three_elements, 3.2.1-02_generation_typed_prenorm, 3.2.1-05_generation_prov_role, 3.2.1-07_no_time, 3.2.1-09_full_provenance, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time, 3.2.7-03_revision_type, 3.2.9-03_with_role, A.1-01_spec_example42, A.2-01_spec_example43</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>2.2-01_spec_example1_typed, 2.2-02_lang_tagged_string, 2.2-09_single_typed_custom_attr, 2.2-13_prov_type_qualified_name, 2.2-14_prov_location_typed, 2.2-17_empty_string_value, 2.2-18_custom_type, 2.2-24_prov_label_single_lang, 2.2-25_mixed_prov_and_custom_attrs, 2.2-27_typed_xsd_string_vs_native, 3.1.1-04_all_prov_attrs, 3.1.1-05_many_custom_attrs, 3.1.1-06_collection_entity, 3.1.1-09_long_entity_id, 3.1.1-10_entity_with_activity_agent, 3.1.1-17_two_prov_types, 3.1.1-19_prov_type_typed_string, 3.1.1-21_entity_only_no_other_sections, 3.1.2-02_agent_typed_attrs, 3.1.2-04_agent_prov_label, 3.1.2-05_agent_prov_location, 3.1.2-09_agent_plus_entity, 3.1.2-15_agent_label_lang, 3.1.3-02_activity_typed_attrs, 3.1.3-05_no_times, 3.1.3-09_all_three_elements, 3.2.1-02_generation_typed_prenorm, 3.2.1-05_generation_prov_role, 3.2.1-07_no_time, 3.2.1-09_full_provenance, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time, 3.2.7-03_revision_type, 3.2.9-03_with_role, A.1-01_spec_example42, A.2-01_spec_example43</t>
+          <t>POST-PROCESS OUTPUT: Convert [type, value] arrays to {"$": value, "type": type} objects.</t>
         </is>
       </c>
     </row>
@@ -11067,32 +11025,27 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Native strings in an array survive:
-  Input:  "ex:tags": ["alpha", "beta", "gamma"]
-  Output: "ex:tags": ["beta", "alpha", "gamma"]  — present but reordered</t>
+          <t>Native strings behave differently depending on context — dropped when alone, kept in arrays</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>A native string as sole value is dropped (D2.2-2):
-  Input:  "ex:name": "hello"
-  Output: entity becomes { }  — attribute gone
-Same data type, same spec permission. The only difference is whether it is the sole value or one of many in an array.</t>
+          <t>Spec §2.2 allows native types equally in both contexts; inconsistent handling</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>Spec Section 2.2</t>
+          <t>2.2-19_native_string_array</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>2.2-19_native_string_array</t>
+          <t>PRE-PROCESS: Same as D2.2-2 - always use typed format for all values.</t>
         </is>
       </c>
     </row>
@@ -11104,24 +11057,25 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>2-element array output has non-deterministic element order</t>
+        </is>
+      </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>The [value, type] arrays from D2.2-1 do not have consistent element order. From the SAME test, SAME entity:
-  "ex:byteSize"    -&gt; ["xsd:positiveInteger", "1034"]     (type first)
-  "ex:compression" -&gt; ["82.5e-2", "xsd:double"]           (value first)
-The order depends on Java's internal hash codes for the strings. So a consumer cannot even rely on position to tell value from type.</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>Spec Section 2.2</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr"/>
+          <t>The `[value, type]` arrays from D2.2-1 have unpredictable element order depending on Java hash codes, making the already-incorrect format additionally unreliable</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr"/>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>POST-PROCESS: Same as D2.2-1. Detect type vs value by colon in qualified name.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -11131,36 +11085,27 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>On entities, prov:value partially works (key survives, content often lost — see D2.2-5).</t>
+          <t>`prov:value` completely dropped on Agent elements</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>On agents and activities, the ENTIRE prov:value attribute disappears:
-  Entity input:   "prov:value": {"$":"42","type":"xsd:int"}
-  Entity output:  "prov:value": ["xsd:int"]  — key survives, content lost
-  Agent input:    "prov:value": {"$":"agent-data-123","type":"xsd:string"}
-  Agent output:   "ex:ag1": { }  — ENTIRE attribute gone
-  Agent input:    "prov:value": {"$":"42","type":"xsd:int"}
-  Agent output:   "ex:ag1": { }  — ENTIRE attribute gone
-  Activity input: "prov:value": {"$":"computation-result","type":"xsd:string"}
-  Activity output: "ex:a1": { }  — ENTIRE attribute gone
-Tests: 3.1.2-06, 3.1.2-13 (agents), 3.1.3-07 (activity).</t>
+          <t>`prov:value` is a defined PROV-DM attribute for elements; read in but not written back out on agents specifically</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>PROV-DM attribute definition</t>
+          <t>3.1.2-06_agent_prov_value, 3.1.2-13_agent_prov_value_int, 3.1.3-07_activity_prov_value</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>3.1.2-06_agent_prov_value, 3.1.2-13_agent_prov_value_int, 3.1.3-07_activity_prov_value</t>
+          <t>Same as D2.2-5: Rename "prov:value" to custom attribute, rename back after.</t>
         </is>
       </c>
     </row>
@@ -11172,30 +11117,27 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>A single typed value on an agent keeps its type (as wrong array format).</t>
+          <t>Multi-value `xsd:string` attributes lose type annotation</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Two or more xsd:string values on the same attribute — type stripped:
-  Input:  "ex:role": [{"$":"developer","type":"xsd:string"}, {"$":"manager","type":"xsd:string"}]
-  Output: "ex:role": ["developer", "manager"]
-Values survive. Type annotations gone. You cannot tell if these were typed xsd:string or plain native strings.</t>
+          <t>When an agent has ≥2 `xsd:string` typed values, the type information is stripped from the output; values survive but lose their type</t>
         </is>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>Spec Section 2.2</t>
+          <t>3.1.2-10_agent_multivalue_attr</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>3.1.2-10_agent_multivalue_attr</t>
+          <t>POST-PROCESS: Re-wrap bare strings with {"$": "value", "type": "xsd:string"} when original had typed format.</t>
         </is>
       </c>
     </row>
@@ -11207,33 +11149,27 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Pre-formatted timestamps matching ProvToolbox's own output format round-trip perfectly. Test 3.1.3-13 passes with "2011-11-16T16:05:00.000+01:00".</t>
+          <t>Timestamps silently modified — timezone injected, milliseconds added, sub-ms truncated</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>Any other valid xsd:dateTime format is modified:
-  "2011-11-16T16:05:00"        -&gt; "2011-11-16T16:05:00.000+01:00"  (added .000 and local TZ)
-  "2011-11-16T16:05:00Z"       -&gt; "2011-11-16T16:05:00.000Z"       (added .000)
-  "2011-11-16T16:06:00.456789Z"-&gt; "2011-11-16T16:06:00.456Z"       (truncated microseconds)
-  "2011-11-16" (date only)     -&gt; "2011-11-16T00:00:00.000+01:00"  (added time, ms, local TZ)
-The +01:00 is the MACHINE'S LOCAL TIMEZONE — same input produces different output depending on where you run it. Adding a timezone changes semantic meaning: "unspecified timezone" becomes "explicitly UTC+1".
-Tests: 3.1.3-01 through 3.1.3-12 (except 3.1.3-13 which passes), 3.1.3-14.</t>
+          <t>Spec §3.1.3: timestamps "**MUST** conform to xsd:dateTime" — the spec does not explicitly require preserving the exact lexical form. However, injecting `+00:00` changes semantic meaning: a timezone-unspecified value becomes explicitly UTC. Spec Example 9 shows timestamps without timezone or milliseconds</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>Spec Section 3.1.3, Example 9</t>
+          <t>3.1.3-01_spec_example9, 3.1.3-02_activity_typed_attrs, 3.1.3-03_start_time_only, 3.1.3-04_end_time_only, 3.1.3-06_multiple_activities, 3.1.3-09_all_three_elements, 3.1.3-10_time_precision, 3.1.3-14_time_date_only, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>3.1.3-01_spec_example9, 3.1.3-02_activity_typed_attrs, 3.1.3-03_start_time_only, 3.1.3-04_end_time_only, 3.1.3-06_multiple_activities, 3.1.3-09_all_three_elements, 3.1.3-10_time_precision, 3.1.3-14_time_date_only, 3.2.1-01_spec_example11, 3.2.2-01_spec_example13</t>
+          <t>PRE/POST-PROCESS: Store original timestamps, restore after round-trip. Or accept normalized format.</t>
         </is>
       </c>
     </row>
@@ -11245,30 +11181,27 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>Single values stay in place.</t>
+          <t>Multi-value array order not preserved</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Multi-value arrays get reordered:
-  Input:  ["alpha", "beta", "gamma"]
-  Output: ["beta", "alpha", "gamma"]
-Content survives, order does not. Array order is semantically significant in JSON, but the spec does not explicitly require preserving it.</t>
+          <t>Spec §2.2: multiple values "**MUST** be... collated in to a JSON array." Array order is semantically significant in JSON, but the spec does not explicitly require preserving it</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>Spec Section 2.2</t>
+          <t>2.2-10_array_typed_values, 2.2-11_multiple_lang_tags, 3.1.1-13_multiple_prov_types, 3.1.2-14_agent_multivalue_qname</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>2.2-10_array_typed_values, 2.2-11_multiple_lang_tags, 3.1.1-13_multiple_prov_types, 3.1.2-14_agent_multivalue_qname</t>
+          <t>Accept or POST-PROCESS to re-sort arrays in deterministic order.</t>
         </is>
       </c>
     </row>
@@ -11280,30 +11213,27 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Data within each element is complete.</t>
+          <t>Element order within sections not preserved</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Element ordering within sections changes:
-  Input order:  "ex:e1", "ex:e2", "ex:e3"
-  Output order: may become "ex:e3", "ex:e1", "ex:e2"
-JSON object key order is not guaranteed by the JSON spec, so this is debatable, but many systems depend on it in practice.</t>
+          <t>JSON object key order is not guaranteed by the JSON specification; however many systems depend on it in practice</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>JSON specification</t>
+          <t>3.1.1-03_multiple_entities, 3.1.2-03_multiple_agents, 3.1.3-06_multiple_activities, 3.2.1-08_multiple_generations</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>3.1.1-03_multiple_entities, 3.1.2-03_multiple_agents, 3.1.3-06_multiple_activities, 3.2.1-08_multiple_generations</t>
+          <t>Accept - JSON object key order is not guaranteed by RFC 8259.</t>
         </is>
       </c>
     </row>
@@ -11315,23 +11245,27 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr"/>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Duplicate JSON keys — last wins silently</t>
+        </is>
+      </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Duplicate JSON keys in the same object — last one wins silently. This is standard JSON parser behaviour per RFC 8259, not specific to ProvToolbox.</t>
+          <t>Standard JSON parser behaviour per RFC 8259; not specific to ProvToolbox</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>RFC 8259</t>
+          <t>3.1.1-08_duplicate_entity_id</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>3.1.1-08_duplicate_entity_id</t>
+          <t>PRE-PROCESS: Validate for duplicate keys. Standard JSON behavior.</t>
         </is>
       </c>
     </row>
@@ -11343,27 +11277,27 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>prov:role on relations (wasGeneratedBy, wasAssociatedWith, etc.) is preserved. Test 3.2.1-05 and 3.2.9-03 show prov:role surviving on relations (wrong array format, but data is there).</t>
+          <t>`prov:role` silently dropped on elements</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>prov:role on elements (entity, agent, activity) is dropped. PROV-DM defines prov:role for relations, not elements, so dropping it on elements is arguably correct — but it could be preserved as a generic attribute.</t>
+          <t>PROV-DM defines `prov:role` for relations, not elements. Elements can have arbitrary additional attributes, so `prov:role` should be preserved as a generic attribute, but it is not a standard element attribute</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>PROV-DM</t>
+          <t>3.1.1-04_all_prov_attrs, 3.1.1-20_prov_role, 3.1.2-07_agent_prov_role, 3.1.3-08_activity_prov_role</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>3.1.1-04_all_prov_attrs, 3.1.1-20_prov_role, 3.1.2-07_agent_prov_role, 3.1.3-08_activity_prov_role</t>
+          <t>PRE-PROCESS: Rename "prov:role" to custom attribute on elements.</t>
         </is>
       </c>
     </row>
@@ -11375,27 +11309,27 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Sections with actual data are always present.</t>
+          <t>Empty statement sections dropped from output</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Empty sections like "entity": {} are dropped from output entirely. No data was in them, so no data is lost. Cosmetic difference only.</t>
+          <t>Spec shows sections containing data; it does not explicitly require preserving empty sections. No data loss</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Spec examples</t>
+          <t>3.1.1-12_empty_entity_section, 3.1.2-08_empty_agent_section, 3.1.3-11_empty_activity_section, 3.2.1-10_empty_wgb_section</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>3.1.1-12_empty_entity_section, 3.1.2-08_empty_agent_section, 3.1.3-11_empty_activity_section, 3.2.1-10_empty_wgb_section</t>
+          <t>Accept - empty sections carry no data. Or POST-PROCESS to add back.</t>
         </is>
       </c>
     </row>
@@ -11407,23 +11341,27 @@
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr"/>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Property order within relation objects changed from input</t>
+        </is>
+      </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>Property order within relation objects is changed from input. For example, "prov:entity" and "prov:activity" keys may swap positions. JSON object key order is not guaranteed. Data is intact, only structure differs.</t>
+          <t>JSON object key order is not guaranteed; data intact but structure differs</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>JSON specification</t>
+          <t>3.2.2-01_spec_example13, 3.2.2-02_named_minimal, 3.2.2-03_anonymous_blank_node, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>3.2.2-01_spec_example13, 3.2.2-02_named_minimal, 3.2.2-03_anonymous_blank_node, 3.2.2-04_usage_prov_role, 3.2.2-05_typed_prenorm_time</t>
+          <t>Accept - JSON key order not guaranteed. No data lost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add developer questions column and update workarounds with verified test results
- New "Questions for Developer" column on both reports asking whether each issue
  is a bug or design choice, with specific questions per issue
- Updated workaround descriptions to reflect actual test verification results
- D3.1.2-2: use xsd:normalizedString to preserve type annotations
- All 19 workarounds tested through ProvToolbox and marked as VERIFIED/POST-PROCESS/ACCEPT
</commit_message>
<xml_diff>
--- a/compatibility_results.xlsx
+++ b/compatibility_results.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Tests'!$A$1:$I$136</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues'!$A$1:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues'!$A$1:$G$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10722,15 +10722,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10761,7 +10762,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Workaround</t>
+          <t>Workaround (Verified)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Questions for Developer</t>
         </is>
       </c>
     </row>
@@ -10793,7 +10799,12 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>PRE-PROCESS INPUT: Convert native JSON values to typed format. "ex:name": "hello" -&gt; "ex:name": [{"$": "hello", "type": "xsd:string"}]</t>
+          <t>VERIFIED: Convert native values to typed format before input. Tested: data survives round-trip.</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Is not supporting native JSON values a deliberate design choice? The spec says "MAY" — does ProvToolbox intentionally only support typed format? Should it throw an error instead of silently dropping?</t>
         </is>
       </c>
     </row>
@@ -10825,7 +10836,12 @@
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>PRE-PROCESS INPUT: Convert native values in arrays to typed format. Eliminates the crash.</t>
+          <t>VERIFIED: Convert all native values in arrays to typed format. Tested: no crash, both values survive.</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Even if native values are not supported, should mixed arrays give a clean error rather than crashing? This is Spec Example 3.</t>
         </is>
       </c>
     </row>
@@ -10857,7 +10873,12 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Rename "prov:value" to custom attribute (e.g., "ex:provValue"). POST-PROCESS: Rename back.</t>
+          <t>VERIFIED: Rename "prov:value" to custom attribute (e.g., "ex:provValue"). Tested: data survives.</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Is the @JsonIgnore on getValue() intentional? Is prov:value handled through a separate serialization path?</t>
         </is>
       </c>
     </row>
@@ -10885,7 +10906,12 @@
       <c r="E5" s="15" t="inlineStr"/>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Validate JSON and remove/replace null attribute values before passing to ProvToolbox.</t>
+          <t>VERIFIED: Remove/replace null attribute values before input. Tested: works fine.</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Should the parser handle null gracefully? Should it ignore with a warning rather than crashing?</t>
         </is>
       </c>
     </row>
@@ -10917,7 +10943,12 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>NO IN-FORMAT WORKAROUND. Extract bundle contents into separate documents, or use PROV-N format.</t>
+          <t>VERIFIED: Extract bundle contents as separate documents. Tested: ROUND_TRIP_IDENTICAL. Alternative: PROV-N format.</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Is PROV-JSON bundle support known to be broken or work-in-progress? The NPE is in SortedBundle.toBundle() where this.id is null.</t>
         </is>
       </c>
     </row>
@@ -10949,7 +10980,12 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>NO IN-FORMAT WORKAROUND. Model as regular entities or use PROV-N format.</t>
+          <t>VERIFIED: Model dictionary operations as regular entities. Tested: data survives. Alternative: PROV-N.</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Are PROV-Dictionary extensions intentionally not supported in JSON? Scope limitation or planned feature?</t>
         </is>
       </c>
     </row>
@@ -10981,7 +11017,12 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Avoid "_" as namespace prefix. Rename to "u" or "bnk" in prefix section and all qualified names.</t>
+          <t>VERIFIED: Rename "_" prefix to something else (e.g., "u"). Tested: survives correctly.</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Is the "_" prefix reservation for blank nodes a deliberate design choice? Is it intentional that users cannot use "_" as a namespace prefix?</t>
         </is>
       </c>
     </row>
@@ -11013,7 +11054,12 @@
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>POST-PROCESS OUTPUT: Convert [type, value] arrays to {"$": value, "type": type} objects.</t>
+          <t>POST-PROCESS: Convert [type, value] arrays to {"$":value,"type":type} objects. Tested: data present.</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Is the [type, value] array format a deliberate alternative? Is there documentation for this format?</t>
         </is>
       </c>
     </row>
@@ -11045,7 +11091,12 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Same as D2.2-2 - always use typed format for all values.</t>
+          <t>VERIFIED: Use typed format for all values (same as D2.2-2). Both produce same output for arrays.</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>Is the inconsistency (strings survive in arrays but dropped as sole values) a known side effect of D2.2-2?</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11124,12 @@
       <c r="E11" s="16" t="inlineStr"/>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>POST-PROCESS: Same as D2.2-1. Detect type vs value by colon in qualified name.</t>
+          <t>POST-PROCESS: Same as D2.2-1. Detect type vs value by colon in qualified name pattern.</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Is the element order within [type, value] arrays expected to be stable? Is HashMap iteration order depended on?</t>
         </is>
       </c>
     </row>
@@ -11105,7 +11161,12 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Same as D2.2-5: Rename "prov:value" to custom attribute, rename back after.</t>
+          <t>VERIFIED: Rename "prov:value" to custom attribute. Tested: data survives.</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Same as D2.2-5 — is there a reason prov:value is treated differently from prov:label and prov:type?</t>
         </is>
       </c>
     </row>
@@ -11137,7 +11198,12 @@
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>POST-PROCESS: Re-wrap bare strings with {"$": "value", "type": "xsd:string"} when original had typed format.</t>
+          <t>VERIFIED: Use xsd:normalizedString instead of xsd:string. Tested: type annotation preserved.</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Is stripping xsd:string type annotation intentional for readability? By design to produce cleaner JSON?</t>
         </is>
       </c>
     </row>
@@ -11169,7 +11235,12 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>PRE/POST-PROCESS: Store original timestamps, restore after round-trip. Or accept normalized format.</t>
+          <t>POST-PROCESS: Store original timestamps before round-trip, restore after. Tested: data present but modified.</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Is DateTimeOption.PRESERVE supposed to keep the original format? Is there a way to get unmodified timestamps? Is timezone injection configurable?</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11272,12 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>Accept or POST-PROCESS to re-sort arrays in deterministic order.</t>
+          <t>Accept or post-process to re-sort. Tested: order was preserved in this case.</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Is preserving array order a goal? Could LinkedHashSet be used instead of HashSet?</t>
         </is>
       </c>
     </row>
@@ -11233,7 +11309,12 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>Accept - JSON object key order is not guaranteed by RFC 8259.</t>
+          <t>Accept - JSON object key order is not guaranteed by RFC 8259. Tested: data intact.</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>Is HashMap (unordered) intentional? Would LinkedHashMap preserve insertion order?</t>
         </is>
       </c>
     </row>
@@ -11265,7 +11346,12 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Validate for duplicate keys. Standard JSON behavior.</t>
+          <t>Accept - standard JSON parser behavior (last wins). Tested: last definition survives.</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>Standard behavior. Could ProvToolbox detect and warn about duplicate keys?</t>
         </is>
       </c>
     </row>
@@ -11297,7 +11383,12 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>PRE-PROCESS: Rename "prov:role" to custom attribute on elements.</t>
+          <t>VERIFIED: Rename "prov:role" to custom attribute on elements. Tested: "ex:role" survives.</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Is dropping prov:role on elements intentional? Should unknown prov: attributes be preserved as generic attributes?</t>
         </is>
       </c>
     </row>
@@ -11329,7 +11420,12 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Accept - empty sections carry no data. Or POST-PROCESS to add back.</t>
+          <t>Accept - empty sections carry no data. Tested: section dropped, no data loss.</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>Is @JsonInclude(NON_EMPTY) intentional to keep output clean? Should empty sections be preserved?</t>
         </is>
       </c>
     </row>
@@ -11361,12 +11457,17 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Accept - JSON key order not guaranteed. No data lost.</t>
+          <t>Accept - JSON key order not guaranteed. Tested: all properties and values intact.</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Standard JSON behavior. Is there a @JsonPropertyOrder for consistent ordering?</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F20"/>
+  <autoFilter ref="A1:G20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>